<commit_message>
fix: add fechaContrato to clean test Excels, improve ProcessRail navigation, remove redundant traceability panel
- Add FECHA DE CONTRATO to all 3 clean Excel META rows (fixes XML validation error)
- ProcessRail: active step takes precedence over done state so current phase is always highlighted
- ProcessRail: consolidated step (4) navigates back to review instead of re-consolidating
- Remove TraceabilityPanel (redundant with ProcessRail)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/test1-clean.xlsx
+++ b/test-data/test1-clean.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,26 +434,26 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>FECHA DE ENTRADA</v>
+        <v>FECHA DE CONTRATO</v>
       </c>
       <c r="B7" t="str">
-        <v>01/06/2024</v>
+        <v>15/05/2024</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>FECHA DE SALIDA</v>
+        <v>FECHA DE ENTRADA</v>
       </c>
       <c r="B8" t="str">
-        <v>08/06/2024</v>
+        <v>01/06/2024</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>HORA</v>
+        <v>FECHA DE SALIDA</v>
       </c>
       <c r="B9" t="str">
-        <v>15:00</v>
+        <v>08/06/2024</v>
       </c>
     </row>
     <row r="10">
@@ -461,131 +461,92 @@
         <v>HORA</v>
       </c>
       <c r="B10" t="str">
-        <v>11:00</v>
+        <v>15:00</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>NUMERO DE PERSONAS</v>
+        <v>HORA</v>
       </c>
       <c r="B11" t="str">
-        <v>7</v>
+        <v>11:00</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>TIPO DE PAGO</v>
+        <v>NUMERO DE PERSONAS</v>
       </c>
       <c r="B12" t="str">
-        <v>TARJETA</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Nombre</v>
+        <v>TIPO DE PAGO</v>
       </c>
       <c r="B13" t="str">
-        <v>1. Apellido</v>
-      </c>
-      <c r="C13" t="str">
-        <v>2. Apellido</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Fecha de nacimiento</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Nationality</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Tipo de documento de identidad</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Número de documento</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Soporte de documento</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Dirección de residencia</v>
-      </c>
-      <c r="J13" t="str">
-        <v>Código municipio</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Correo electrónico</v>
-      </c>
-      <c r="L13" t="str">
-        <v>Número de teléfono</v>
-      </c>
-      <c r="M13" t="str">
-        <v>Fecha de llegada</v>
-      </c>
-      <c r="N13" t="str">
-        <v>Fecha de salida</v>
-      </c>
-      <c r="O13" t="str">
-        <v>Parentesco</v>
+        <v>TARJETA</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>María</v>
+        <v>Nombre</v>
       </c>
       <c r="B14" t="str">
-        <v>García</v>
+        <v>1. Apellido</v>
       </c>
       <c r="C14" t="str">
-        <v>López</v>
+        <v>2. Apellido</v>
       </c>
       <c r="D14" t="str">
-        <v>15/03/1985</v>
+        <v>Fecha de nacimiento</v>
       </c>
       <c r="E14" t="str">
-        <v>ESP</v>
+        <v>Nationality</v>
       </c>
       <c r="F14" t="str">
-        <v>NIF</v>
+        <v>Tipo de documento de identidad</v>
       </c>
       <c r="G14" t="str">
-        <v>12345678Z</v>
+        <v>Número de documento</v>
       </c>
       <c r="H14" t="str">
-        <v>AAA111111</v>
+        <v>Soporte de documento</v>
       </c>
       <c r="I14" t="str">
-        <v>Calle Mayor 1, 46812 Riola, Valencia</v>
+        <v>Dirección de residencia</v>
       </c>
       <c r="J14" t="str">
-        <v>46215</v>
+        <v>Código municipio</v>
       </c>
       <c r="K14" t="str">
-        <v>maria@example.com</v>
+        <v>Correo electrónico</v>
       </c>
       <c r="L14" t="str">
-        <v>+34600111222</v>
+        <v>Número de teléfono</v>
       </c>
       <c r="M14" t="str">
-        <v>01/06/2024</v>
+        <v>Fecha de llegada</v>
       </c>
       <c r="N14" t="str">
-        <v>08/06/2024</v>
+        <v>Fecha de salida</v>
       </c>
       <c r="O14" t="str">
-        <v>TI</v>
+        <v>Parentesco</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Pedro</v>
+        <v>María</v>
       </c>
       <c r="B15" t="str">
-        <v>Martínez</v>
+        <v>García</v>
       </c>
       <c r="C15" t="str">
-        <v>Sánchez</v>
+        <v>López</v>
       </c>
       <c r="D15" t="str">
-        <v>22/07/1978</v>
+        <v>15/03/1985</v>
       </c>
       <c r="E15" t="str">
         <v>ESP</v>
@@ -594,10 +555,10 @@
         <v>NIF</v>
       </c>
       <c r="G15" t="str">
-        <v>33445566R</v>
+        <v>12345678Z</v>
       </c>
       <c r="H15" t="str">
-        <v>BBB222222</v>
+        <v>AAA111111</v>
       </c>
       <c r="I15" t="str">
         <v>Calle Mayor 1, 46812 Riola, Valencia</v>
@@ -606,10 +567,10 @@
         <v>46215</v>
       </c>
       <c r="K15" t="str">
-        <v>pedro@example.com</v>
+        <v>maria@example.com</v>
       </c>
       <c r="L15" t="str">
-        <v>+34600333444</v>
+        <v>+34600111222</v>
       </c>
       <c r="M15" t="str">
         <v>01/06/2024</v>
@@ -618,33 +579,33 @@
         <v>08/06/2024</v>
       </c>
       <c r="O15" t="str">
-        <v>OT</v>
+        <v>TI</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Piotr</v>
+        <v>Pedro</v>
       </c>
       <c r="B16" t="str">
-        <v>Kowalski</v>
+        <v>Martínez</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>Sánchez</v>
       </c>
       <c r="D16" t="str">
-        <v>10/05/1990</v>
+        <v>22/07/1978</v>
       </c>
       <c r="E16" t="str">
         <v>ESP</v>
       </c>
       <c r="F16" t="str">
-        <v>NIE</v>
+        <v>NIF</v>
       </c>
       <c r="G16" t="str">
-        <v>X1234567L</v>
+        <v>33445566R</v>
       </c>
       <c r="H16" t="str">
-        <v>CCC333333</v>
+        <v>BBB222222</v>
       </c>
       <c r="I16" t="str">
         <v>Calle Mayor 1, 46812 Riola, Valencia</v>
@@ -653,10 +614,10 @@
         <v>46215</v>
       </c>
       <c r="K16" t="str">
-        <v>piotr@example.com</v>
+        <v>pedro@example.com</v>
       </c>
       <c r="L16" t="str">
-        <v>+34611222333</v>
+        <v>+34600333444</v>
       </c>
       <c r="M16" t="str">
         <v>01/06/2024</v>
@@ -670,28 +631,28 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Ana</v>
+        <v>Piotr</v>
       </c>
       <c r="B17" t="str">
-        <v>Rodríguez</v>
+        <v>Kowalski</v>
       </c>
       <c r="C17" t="str">
-        <v>Pérez</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>08/11/1992</v>
+        <v>10/05/1990</v>
       </c>
       <c r="E17" t="str">
         <v>ESP</v>
       </c>
       <c r="F17" t="str">
-        <v>NIF</v>
+        <v>NIE</v>
       </c>
       <c r="G17" t="str">
-        <v>11223344B</v>
+        <v>X1234567L</v>
       </c>
       <c r="H17" t="str">
-        <v>DDD444444</v>
+        <v>CCC333333</v>
       </c>
       <c r="I17" t="str">
         <v>Calle Mayor 1, 46812 Riola, Valencia</v>
@@ -700,10 +661,10 @@
         <v>46215</v>
       </c>
       <c r="K17" t="str">
-        <v>ana@example.com</v>
+        <v>piotr@example.com</v>
       </c>
       <c r="L17" t="str">
-        <v>+34622333444</v>
+        <v>+34611222333</v>
       </c>
       <c r="M17" t="str">
         <v>01/06/2024</v>
@@ -717,40 +678,40 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Jean</v>
+        <v>Ana</v>
       </c>
       <c r="B18" t="str">
-        <v>Dupont</v>
+        <v>Rodríguez</v>
       </c>
       <c r="C18" t="str">
-        <v>Martin</v>
+        <v>Pérez</v>
       </c>
       <c r="D18" t="str">
-        <v>30/04/1982</v>
+        <v>08/11/1992</v>
       </c>
       <c r="E18" t="str">
-        <v>FRA</v>
+        <v>ESP</v>
       </c>
       <c r="F18" t="str">
-        <v>PAS</v>
+        <v>NIF</v>
       </c>
       <c r="G18" t="str">
-        <v>12AB34567</v>
+        <v>11223344B</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>DDD444444</v>
       </c>
       <c r="I18" t="str">
-        <v>14 Rue de la Paix, Lyon, 69001</v>
+        <v>Calle Mayor 1, 46812 Riola, Valencia</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>46215</v>
       </c>
       <c r="K18" t="str">
-        <v>jean@example.com</v>
+        <v>ana@example.com</v>
       </c>
       <c r="L18" t="str">
-        <v>+33600112233</v>
+        <v>+34622333444</v>
       </c>
       <c r="M18" t="str">
         <v>01/06/2024</v>
@@ -764,40 +725,40 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Hans</v>
+        <v>Jean</v>
       </c>
       <c r="B19" t="str">
-        <v>Müller</v>
+        <v>Dupont</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>Martin</v>
       </c>
       <c r="D19" t="str">
-        <v>18/09/1975</v>
+        <v>30/04/1982</v>
       </c>
       <c r="E19" t="str">
-        <v>DEU</v>
+        <v>FRA</v>
       </c>
       <c r="F19" t="str">
         <v>PAS</v>
       </c>
       <c r="G19" t="str">
-        <v>C3T9L5K21</v>
+        <v>12AB34567</v>
       </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>Hauptstraße 42, Berlin, 10115</v>
+        <v>14 Rue de la Paix, Lyon, 69001</v>
       </c>
       <c r="J19" t="str">
         <v/>
       </c>
       <c r="K19" t="str">
-        <v>hans@example.com</v>
+        <v>jean@example.com</v>
       </c>
       <c r="L19" t="str">
-        <v>+49151234567</v>
+        <v>+33600112233</v>
       </c>
       <c r="M19" t="str">
         <v>01/06/2024</v>
@@ -811,40 +772,40 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Giulia</v>
+        <v>Hans</v>
       </c>
       <c r="B20" t="str">
-        <v>Rossi</v>
+        <v>Müller</v>
       </c>
       <c r="C20" t="str">
-        <v>Ferrari</v>
+        <v/>
       </c>
       <c r="D20" t="str">
-        <v>05/02/1988</v>
+        <v>18/09/1975</v>
       </c>
       <c r="E20" t="str">
-        <v>ITA</v>
+        <v>DEU</v>
       </c>
       <c r="F20" t="str">
-        <v>OTRO</v>
+        <v>PAS</v>
       </c>
       <c r="G20" t="str">
-        <v>CA12345AA</v>
+        <v>C3T9L5K21</v>
       </c>
       <c r="H20" t="str">
         <v/>
       </c>
       <c r="I20" t="str">
-        <v>Via Roma 7, Milano, 20100</v>
+        <v>Hauptstraße 42, Berlin, 10115</v>
       </c>
       <c r="J20" t="str">
         <v/>
       </c>
       <c r="K20" t="str">
-        <v>giulia@example.com</v>
+        <v>hans@example.com</v>
       </c>
       <c r="L20" t="str">
-        <v>+39333111222</v>
+        <v>+49151234567</v>
       </c>
       <c r="M20" t="str">
         <v>01/06/2024</v>
@@ -856,9 +817,56 @@
         <v>OT</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Giulia</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Rossi</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Ferrari</v>
+      </c>
+      <c r="D21" t="str">
+        <v>05/02/1988</v>
+      </c>
+      <c r="E21" t="str">
+        <v>ITA</v>
+      </c>
+      <c r="F21" t="str">
+        <v>OTRO</v>
+      </c>
+      <c r="G21" t="str">
+        <v>CA12345AA</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>Via Roma 7, Milano, 20100</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v>giulia@example.com</v>
+      </c>
+      <c r="L21" t="str">
+        <v>+39333111222</v>
+      </c>
+      <c r="M21" t="str">
+        <v>01/06/2024</v>
+      </c>
+      <c r="N21" t="str">
+        <v>08/06/2024</v>
+      </c>
+      <c r="O21" t="str">
+        <v>OT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align SES test fixtures with preproduction credentials
</commit_message>
<xml_diff>
--- a/test-data/test1-clean.xlsx
+++ b/test-data/test1-clean.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,7 +401,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>CODIGO 12345</v>
+        <v>CODIGO 0000004630</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
fix: reject fechaEntrada > 1 year old locally and update test data dates to 2026
SES server rejects check-in dates more than 1 year in the past. Added the same
rule to the local validator so it surfaces before the SOAP round-trip.
Updated test1-clean.xlsx dates from June 2024 to April/May 2026.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/test1-clean.xlsx
+++ b/test-data/test1-clean.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -437,7 +437,7 @@
         <v>FECHA DE CONTRATO</v>
       </c>
       <c r="B7" t="str">
-        <v>15/05/2024</v>
+        <v>20/04/2026</v>
       </c>
     </row>
     <row r="8">
@@ -445,7 +445,7 @@
         <v>FECHA DE ENTRADA</v>
       </c>
       <c r="B8" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
     </row>
     <row r="9">
@@ -453,7 +453,7 @@
         <v>FECHA DE SALIDA</v>
       </c>
       <c r="B9" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
     </row>
     <row r="10">
@@ -573,10 +573,10 @@
         <v>+34600111222</v>
       </c>
       <c r="M15" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N15" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O15" t="str">
         <v>TI</v>
@@ -620,10 +620,10 @@
         <v>+34600333444</v>
       </c>
       <c r="M16" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N16" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O16" t="str">
         <v>OT</v>
@@ -667,10 +667,10 @@
         <v>+34611222333</v>
       </c>
       <c r="M17" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N17" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O17" t="str">
         <v>OT</v>
@@ -714,10 +714,10 @@
         <v>+34622333444</v>
       </c>
       <c r="M18" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N18" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O18" t="str">
         <v>OT</v>
@@ -761,10 +761,10 @@
         <v>+33600112233</v>
       </c>
       <c r="M19" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N19" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O19" t="str">
         <v>OT</v>
@@ -808,10 +808,10 @@
         <v>+49151234567</v>
       </c>
       <c r="M20" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N20" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O20" t="str">
         <v>OT</v>
@@ -855,10 +855,10 @@
         <v>+39333111222</v>
       </c>
       <c r="M21" t="str">
-        <v>01/06/2024</v>
+        <v>25/04/2026</v>
       </c>
       <c r="N21" t="str">
-        <v>08/06/2024</v>
+        <v>02/05/2026</v>
       </c>
       <c r="O21" t="str">
         <v>OT</v>

</xml_diff>